<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table40, economy-table42-44
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table40.xlsx
+++ b/sources/table_normalization/xlsx/economy-table40.xlsx
@@ -1056,7 +1056,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1125,12 +1125,6 @@
     <xf numFmtId="15" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1144,9 +1138,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1177,6 +1168,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1485,7 +1488,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1497,325 +1500,330 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="8" max="8" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="11.453125" customWidth="1"/>
+    <col min="10" max="10" width="14.6328125" customWidth="1"/>
     <col min="12" max="12" width="12.453125" customWidth="1"/>
+    <col min="13" max="13" width="15.81640625" customWidth="1"/>
     <col min="14" max="14" width="30.6328125" customWidth="1"/>
     <col min="17" max="17" width="13" customWidth="1"/>
     <col min="18" max="18" width="12.36328125" customWidth="1"/>
     <col min="19" max="19" width="14.7265625" customWidth="1"/>
     <col min="20" max="20" width="11.7265625" customWidth="1"/>
+    <col min="30" max="30" width="13.1796875" customWidth="1"/>
+    <col min="41" max="41" width="11.90625" customWidth="1"/>
+    <col min="42" max="42" width="12.26953125" customWidth="1"/>
+    <col min="44" max="44" width="11.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:73">
-      <c r="A1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="28" t="s">
+      <c r="A1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="27" t="s">
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27" t="s">
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="27"/>
-      <c r="Y1" s="27"/>
-      <c r="Z1" s="27"/>
-      <c r="AA1" s="28" t="s">
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
+      <c r="AA1" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="28"/>
-      <c r="AD1" s="27" t="s">
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
+      <c r="AD1" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="AE1" s="27"/>
-      <c r="AF1" s="27"/>
-      <c r="AG1" s="27"/>
-      <c r="AH1" s="27"/>
-      <c r="AI1" s="27"/>
-      <c r="AJ1" s="27" t="s">
+      <c r="AE1" s="42"/>
+      <c r="AF1" s="42"/>
+      <c r="AG1" s="42"/>
+      <c r="AH1" s="42"/>
+      <c r="AI1" s="42"/>
+      <c r="AJ1" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="AK1" s="27"/>
-      <c r="AL1" s="27"/>
-      <c r="AM1" s="27"/>
-      <c r="AN1" s="27"/>
-      <c r="AO1" s="28" t="s">
+      <c r="AK1" s="42"/>
+      <c r="AL1" s="42"/>
+      <c r="AM1" s="42"/>
+      <c r="AN1" s="42"/>
+      <c r="AO1" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="AP1" s="28"/>
-      <c r="AQ1" s="28"/>
-      <c r="AR1" s="28"/>
-      <c r="AS1" s="34" t="s">
+      <c r="AP1" s="43"/>
+      <c r="AQ1" s="43"/>
+      <c r="AR1" s="43"/>
+      <c r="AS1" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="AT1" s="34"/>
-      <c r="AU1" s="34"/>
-      <c r="AV1" s="34"/>
-      <c r="AW1" s="34"/>
-      <c r="AX1" s="34"/>
-      <c r="AY1" s="34"/>
-      <c r="AZ1" s="34"/>
-      <c r="BA1" s="34"/>
-      <c r="BB1" s="34"/>
-      <c r="BC1" s="34"/>
-      <c r="BD1" s="34"/>
-      <c r="BE1" s="34"/>
-      <c r="BF1" s="34"/>
-      <c r="BG1" s="34" t="s">
+      <c r="AT1" s="44"/>
+      <c r="AU1" s="44"/>
+      <c r="AV1" s="44"/>
+      <c r="AW1" s="44"/>
+      <c r="AX1" s="44"/>
+      <c r="AY1" s="44"/>
+      <c r="AZ1" s="44"/>
+      <c r="BA1" s="44"/>
+      <c r="BB1" s="44"/>
+      <c r="BC1" s="44"/>
+      <c r="BD1" s="44"/>
+      <c r="BE1" s="44"/>
+      <c r="BF1" s="44"/>
+      <c r="BG1" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="BH1" s="34"/>
-      <c r="BI1" s="34"/>
-      <c r="BJ1" s="34"/>
-      <c r="BK1" s="34"/>
-      <c r="BL1" s="34"/>
-      <c r="BM1" s="34"/>
-      <c r="BN1" s="34"/>
-      <c r="BO1" s="34"/>
-      <c r="BP1" s="34"/>
-      <c r="BQ1" s="34"/>
-      <c r="BR1" s="34"/>
-      <c r="BS1" s="34"/>
-      <c r="BT1" s="34"/>
+      <c r="BH1" s="44"/>
+      <c r="BI1" s="44"/>
+      <c r="BJ1" s="44"/>
+      <c r="BK1" s="44"/>
+      <c r="BL1" s="44"/>
+      <c r="BM1" s="44"/>
+      <c r="BN1" s="44"/>
+      <c r="BO1" s="44"/>
+      <c r="BP1" s="44"/>
+      <c r="BQ1" s="44"/>
+      <c r="BR1" s="44"/>
+      <c r="BS1" s="44"/>
+      <c r="BT1" s="44"/>
       <c r="BU1" s="1"/>
     </row>
     <row r="2" spans="1:73" ht="48">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="36" t="s">
+      <c r="F2" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="32" t="s">
+      <c r="G2" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="I2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="31" t="s">
+      <c r="J2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="32" t="s">
+      <c r="K2" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="29" t="s">
+      <c r="L2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="30" t="s">
+      <c r="M2" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="N2" s="33" t="s">
+      <c r="N2" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="37" t="s">
+      <c r="O2" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="P2" s="37" t="s">
+      <c r="P2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="Q2" s="38" t="s">
+      <c r="Q2" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="38" t="s">
+      <c r="R2" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="38" t="s">
+      <c r="S2" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="38" t="s">
+      <c r="T2" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="38" t="s">
+      <c r="U2" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="V2" s="38" t="s">
+      <c r="V2" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="W2" s="38" t="s">
+      <c r="W2" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="X2" s="38" t="s">
+      <c r="X2" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="Y2" s="39" t="s">
+      <c r="Y2" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="Z2" s="38" t="s">
+      <c r="Z2" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AA2" s="38" t="s">
+      <c r="AA2" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="AB2" s="38" t="s">
+      <c r="AB2" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="AC2" s="37" t="s">
+      <c r="AC2" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="AD2" s="40" t="s">
+      <c r="AD2" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="AE2" s="32" t="s">
+      <c r="AE2" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="AF2" s="38" t="s">
+      <c r="AF2" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AG2" s="38" t="s">
+      <c r="AG2" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AH2" s="38" t="s">
+      <c r="AH2" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AI2" s="38" t="s">
+      <c r="AI2" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="AJ2" s="41" t="s">
+      <c r="AJ2" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="AK2" s="42" t="s">
+      <c r="AK2" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="AL2" s="42" t="s">
+      <c r="AL2" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="AM2" s="42" t="s">
+      <c r="AM2" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="AN2" s="43" t="s">
+      <c r="AN2" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="AO2" s="42" t="s">
+      <c r="AO2" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="AP2" s="42" t="s">
+      <c r="AP2" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="AQ2" s="42" t="s">
+      <c r="AQ2" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="AR2" s="42" t="s">
+      <c r="AR2" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="AS2" s="42" t="s">
+      <c r="AS2" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="AT2" s="42" t="s">
+      <c r="AT2" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="AU2" s="42" t="s">
+      <c r="AU2" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="AV2" s="42" t="s">
+      <c r="AV2" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="AW2" s="42" t="s">
+      <c r="AW2" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="AX2" s="44" t="s">
+      <c r="AX2" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="AY2" s="42" t="s">
+      <c r="AY2" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="AZ2" s="42" t="s">
+      <c r="AZ2" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="BA2" s="42" t="s">
+      <c r="BA2" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="BB2" s="42" t="s">
+      <c r="BB2" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="BC2" s="42" t="s">
+      <c r="BC2" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="BD2" s="42" t="s">
+      <c r="BD2" s="45" t="s">
         <v>65</v>
       </c>
-      <c r="BE2" s="42" t="s">
+      <c r="BE2" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="BF2" s="42" t="s">
+      <c r="BF2" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="BG2" s="42" t="s">
+      <c r="BG2" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="BH2" s="42" t="s">
+      <c r="BH2" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="BI2" s="42" t="s">
+      <c r="BI2" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="BJ2" s="42" t="s">
+      <c r="BJ2" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="BK2" s="42" t="s">
+      <c r="BK2" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="BL2" s="42" t="s">
+      <c r="BL2" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="BM2" s="42" t="s">
+      <c r="BM2" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="BN2" s="42" t="s">
+      <c r="BN2" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="BO2" s="42" t="s">
+      <c r="BO2" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="BP2" s="42" t="s">
+      <c r="BP2" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="BQ2" s="42" t="s">
+      <c r="BQ2" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="BR2" s="42" t="s">
+      <c r="BR2" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="BS2" s="42" t="s">
+      <c r="BS2" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="BT2" s="42" t="s">
+      <c r="BT2" s="45" t="s">
         <v>81</v>
       </c>
       <c r="BU2" s="1"/>

</xml_diff>